<commit_message>
Remove Parker Clubb; use client_lists as sole tracker source.
Drop Clubb from HS list, JSON, and PDF; arb/FA/watch Excel files live in
apexstats/client_lists for site and CI (no Desktop dependency).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/client_lists/HSList.xlsx
+++ b/client_lists/HSList.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,93 +549,93 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clubb, Parker</t>
+          <t>Dyett, Evan</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C/RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mulvane HS (KS)</t>
+          <t>Spruce Creek HS (FL)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>South Carolina</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ks/mulvane/mulvane-wildcats/athletes/parker-clubb/baseball/stats/?careerid=ab3rbm346t988&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/fl/port-orange/spruce-creek-hawks/athletes/evan-dyett/baseball/stats/?careerid=opn0vfku7ld33&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>45795</v>
+        <v>45975</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dyett, Evan</t>
+          <t>Escalante, Jake</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>LHP/OF</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Spruce Creek HS (FL)</t>
+          <t>Soquel HS (CA)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>South Carolina</t>
+          <t>Cal State Fullerton</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/fl/port-orange/spruce-creek-hawks/athletes/evan-dyett/baseball/stats/?careerid=opn0vfku7ld33&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/soquel/soquel-knights/athletes/jake-escalante/baseball/stats/?careerid=j4rj8b8jr68j3&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>45975</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Escalante, Jake</t>
+          <t>Flora, Hudson</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LHP/OF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Soquel HS (CA)</t>
+          <t>Foothill HS (CA)</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -643,7 +643,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Cal State Fullerton</t>
+          <t>UC Santa Barbara</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -653,27 +653,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/soquel/soquel-knights/athletes/jake-escalante/baseball/stats/?careerid=j4rj8b8jr68j3&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/hudson-flora/baseball/stats/?careerid=sr9pkpb394k55&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46145</v>
+        <v>45987</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Flora, Hudson</t>
+          <t xml:space="preserve">Garcia, Gavin </t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Foothill HS (CA)</t>
+          <t>Cajon HS (CA)</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>UC Santa Barbara</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -691,65 +691,61 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/hudson-flora/baseball/stats/?careerid=sr9pkpb394k55&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/san-bernardino/cajon-cowboys/athletes/gavin-garcia/baseball/stats/?careerid=mi14lap9ejc44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45987</v>
+        <v>46012</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Garcia, Gavin </t>
+          <t>Gluting, Tyler</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cajon HS (CA)</t>
+          <t>Metea Valley HS (IL)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>Oklahoma</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AK</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/ca/san-bernardino/cajon-cowboys/athletes/gavin-garcia/baseball/stats/?careerid=mi14lap9ejc44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
-        </is>
-      </c>
+          <t>JF</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" s="2" t="n">
-        <v>46012</v>
+        <v>46256</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gluting, Tyler</t>
+          <t>Haggerty, Will</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metea Valley HS (IL)</t>
+          <t>Moses Brown School (RI)</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -757,23 +753,23 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" s="2" t="n">
-        <v>46256</v>
+        <v>45970</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Haggerty, Will</t>
+          <t>Hirschkorn, Jensen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -783,121 +779,125 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Moses Brown School (RI)</t>
+          <t>Kingsburg HS (CA)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>LSU</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TJ</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>AK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.maxpreps.com/ca/kingsburg/kingsburg-vikings/athletes/jensen-hirschkorn/baseball/stats/?careerid=nl0cjhntsf600&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n">
-        <v>45970</v>
+        <v>46010</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hirschkorn, Jensen</t>
+          <t>Kearney, Aiden</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>INF</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kingsburg HS (CA)</t>
+          <t>Hagerty HS (FL)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LSU</t>
+          <t>Uncommitted</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/kingsburg/kingsburg-vikings/athletes/jensen-hirschkorn/baseball/stats/?careerid=nl0cjhntsf600&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/fl/oviedo/hagerty-huskies/athletes/a-kearney/baseball/stats/?careerid=0g5aokuemta66&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>46010</v>
+        <v>45775</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kearney, Aiden</t>
+          <t>Leeper, Jack</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>INF</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hagerty HS (FL)</t>
+          <t>St. Francis HS (CA)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Uncommitted</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TJ</t>
+          <t>AK/AR</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/fl/oviedo/hagerty-huskies/athletes/a-kearney/baseball/stats/?careerid=0g5aokuemta66&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/mountain-view/saint-francis-lancers/athletes/jack-leeper/baseball/stats/?careerid=4v4p963v8c3td&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>45775</v>
+        <v>45673</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Leeper, Jack</t>
+          <t>Maxon, Matt</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP/OF</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>St. Francis HS (CA)</t>
+          <t>Carmel HS (CA)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -911,103 +911,99 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/mountain-view/saint-francis-lancers/athletes/jack-leeper/baseball/stats/?careerid=4v4p963v8c3td&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/carmel/carmel-padres/athletes/matt-maxon/baseball/stats/?careerid=rl4qkpr1si222&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>45673</v>
+        <v>45946</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Maxon, Matt</t>
+          <t>McMillan, Gavin</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RHP/OF</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Carmel HS (CA)</t>
+          <t>Monte Vista HS (CA)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t xml:space="preserve">Mississippi </t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AK/AR</t>
+          <t xml:space="preserve">PC </t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/carmel/carmel-padres/athletes/matt-maxon/baseball/stats/?careerid=rl4qkpr1si222&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/danville/monte-vista-mustangs/athletes/gavin-mcmillan/baseball/stats/?careerid=cr698s8csjkl5&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>45946</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>McMillan, Gavin</t>
+          <t>Messey, Drew</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>INF</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Monte Vista HS (CA)</t>
+          <t>Westminster Academy (MO)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mississippi </t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PC </t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/ca/danville/monte-vista-mustangs/athletes/gavin-mcmillan/baseball/stats/?careerid=cr698s8csjkl5&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
-        </is>
-      </c>
+          <t>JF</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" s="2" t="n">
-        <v>45841</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Messey, Drew</t>
+          <t>Morris, Josiah</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INF</t>
+          <t>INF/C</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Westminster Academy (MO)</t>
+          <t>Clayton Valley Charter (CA)</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1015,75 +1011,75 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Oklahoma State</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK/AR</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" s="2" t="n">
-        <v>45686</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Morris, Josiah</t>
+          <t>Moylan, Seamus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>INF/C</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Clayton Valley Charter (CA)</t>
+          <t>Spruce Creek HS (FL)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oklahoma State</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AK/AR</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" s="2" t="n">
-        <v>45833</v>
+        <v>45708</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Moylan, Seamus</t>
+          <t>Osting, Vaughn</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Spruce Creek HS (FL)</t>
+          <t>Bloomingdale HS (FL)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>East Tenn. State</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1093,31 +1089,31 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" s="2" t="n">
-        <v>45708</v>
+        <v>46120</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Osting, Vaughn</t>
+          <t>Penney, Cam</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>OF/LHP</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bloomingdale HS (FL)</t>
+          <t>Lake Brantley HS (FL)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>East Tenn. State</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1125,33 +1121,37 @@
           <t>TJ</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.maxpreps.com/fl/altamonte-springs/lake-brantley-patriots/athletes/cameron-penney/baseball/stats/?careerid=ggqhvbep14pn7&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="n">
-        <v>46120</v>
+        <v>45972</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Penney, Cam</t>
+          <t>Radwick, Brody</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OF/LHP</t>
+          <t>LHP</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lake Brantley HS (FL)</t>
+          <t>Spurce Creek HS (FL)</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Uncommitted</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1161,127 +1161,127 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/fl/altamonte-springs/lake-brantley-patriots/athletes/cameron-penney/baseball/stats/?careerid=ggqhvbep14pn7&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/fl/port-orange/spruce-creek-hawks/athletes/brody-radwick/baseball/stats/?careerid=bbiiadhmpu2g0&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>45972</v>
+        <v>45727</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Radwick, Brody</t>
+          <t>Saunders, Grady</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LHP</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Spurce Creek HS (FL)</t>
+          <t>Thurston HS (OR)</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Uncommitted</t>
+          <t>Oregon State</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TJ</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/fl/port-orange/spruce-creek-hawks/athletes/brody-radwick/baseball/stats/?careerid=bbiiadhmpu2g0&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
-        </is>
-      </c>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" s="2" t="n">
-        <v>45727</v>
+        <v>45825</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Saunders, Grady</t>
+          <t>Schilling, Jackson</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Thurston HS (OR)</t>
+          <t>Vandalia Butler HS (OH)</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oregon State</t>
+          <t>Ohio State</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>JF</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.maxpreps.com/or/ontario/ontario-tigers/athletes/jackson-schilling/baseball/stats/?careerid=omrlfl01ap255&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="n">
-        <v>45825</v>
+        <v>45909</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Schilling, Jackson</t>
+          <t>Schlicht, Graham</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vandalia Butler HS (OH)</t>
+          <t>De La Salle HS (CA)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ohio State</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>JF</t>
+          <t>AK/AR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/or/ontario/ontario-tigers/athletes/jackson-schilling/baseball/stats/?careerid=omrlfl01ap255&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/concord/de-la-salle-spartans/athletes/graham-schlicht/baseball/stats/?careerid=rp25i2fortsqa&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>45909</v>
+        <v>45855</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Schlicht, Graham</t>
+          <t>Simon, Ryder</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1291,83 +1291,83 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>De La Salle HS (CA)</t>
+          <t>Winter Park HS (FL)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AK/AR</t>
+          <t xml:space="preserve">TJ </t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/concord/de-la-salle-spartans/athletes/graham-schlicht/baseball/stats/?careerid=rp25i2fortsqa&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/fl/winter-park/winter-park-wildcats/athletes/ryder-simon/baseball/stats/?careerid=huv6nf2oal0l5&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>45855</v>
+        <v>45783</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Simon, Ryder</t>
+          <t>Tavares, Aiden</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RHP</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Winter Park HS (FL)</t>
+          <t>Foothill HS (CA)</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t xml:space="preserve">Uncommitted </t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TJ </t>
+          <t>AK/AR</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/fl/winter-park/winter-park-wildcats/athletes/ryder-simon/baseball/stats/?careerid=huv6nf2oal0l5&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/aiden-taveres/baseball/stats/?careerid=bse1ctt9pjfn7&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>45783</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tavares, Aiden</t>
+          <t>Tweedt, Jaxxon</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>OF</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Foothill HS (CA)</t>
+          <t>Chico HS (CA)</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uncommitted </t>
+          <t>Uncommitted</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1385,35 +1385,35 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/pleasanton/foothill-falcons/athletes/aiden-taveres/baseball/stats/?careerid=bse1ctt9pjfn7&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/chico/chico-panthers/athletes/jaxxon-tweedt/baseball/stats/?careerid=h491n4vai4jsc&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46290</v>
+        <v>45894</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tweedt, Jaxxon</t>
+          <t>Vais, Cooper</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OF</t>
+          <t>RHP/OF</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Chico HS (CA)</t>
+          <t>Arvada West HS (CO)</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Uncommitted</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1423,17 +1423,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/chico/chico-panthers/athletes/jaxxon-tweedt/baseball/stats/?careerid=h491n4vai4jsc&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/co/arvada/arvada-west-wildcats/athletes/cooper-vais/baseball/stats/?careerid=si76m65o8fg00&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>45894</v>
+        <v>45995</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Vais, Cooper</t>
+          <t>Whitworth, Tosh</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Arvada West HS (CO)</t>
+          <t>Santa Barbara HS (CA)</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1461,35 +1461,35 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/co/arvada/arvada-west-wildcats/athletes/cooper-vais/baseball/stats/?careerid=si76m65o8fg00&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/santa-barbara/santa-barbara-dons/athletes/tosh-whitworth/baseball/stats/?careerid=l7vhqt67pit44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>45995</v>
+        <v>45899</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Whitworth, Tosh</t>
+          <t>Williams, Brandon</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RHP/OF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Santa Barbara HS (CA)</t>
+          <t>Franklin HS (CA)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>Uncommitted</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1499,17 +1499,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/santa-barbara/santa-barbara-dons/athletes/tosh-whitworth/baseball/stats/?careerid=l7vhqt67pit44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/elk-grove/franklin-wildcats/athletes/brandon-williams/baseball/stats/?careerid=ljhs8khioatdd&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>45899</v>
+        <v>46020</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Williams, Brandon</t>
+          <t>Williams, Gavin</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1519,15 +1519,15 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Franklin HS (CA)</t>
+          <t>Liberty HS (CA)</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Uncommitted</t>
+          <t>Oregon</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1537,27 +1537,27 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/elk-grove/franklin-wildcats/athletes/brandon-williams/baseball/stats/?careerid=ljhs8khioatdd&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/ca/bakersfield/liberty-patriots/athletes/gavin-williams/baseball/stats/?careerid=5eo848nscpq22&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46020</v>
+        <v>45723</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Williams, Gavin</t>
+          <t>Wise, Alex</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>RHP/SS</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Liberty HS (CA)</t>
+          <t>Mount Dora Chrisitian Academy (FL)</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1565,58 +1565,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oregon</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AK/AR</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.maxpreps.com/ca/bakersfield/liberty-patriots/athletes/gavin-williams/baseball/stats/?careerid=5eo848nscpq22&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
+          <t>https://www.maxpreps.com/fl/mount-dora/mount-dora-christian-academy-bulldogs/athletes/alex-wise/baseball/stats/?careerid=1crnqv019sc44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>45723</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Wise, Alex</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>RHP/SS</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Mount Dora Chrisitian Academy (FL)</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>2027</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Auburn</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>TJ</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.maxpreps.com/fl/mount-dora/mount-dora-christian-academy-bulldogs/athletes/alex-wise/baseball/stats/?careerid=1crnqv019sc44&amp;sportSeasonId=1278779e-84df-4e60-8d03-db0024535aa6</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="n">
         <v>46022</v>
       </c>
     </row>

</xml_diff>